<commit_message>
fix(master-excel): Total Hrs formula double-counted OT — now H+L+M
In Payroll_Master_July_2026.xlsx (per-firm salary sheets), the Total Hrs
formula was =H+I+L+M (WorkedHrs + OTHrs + SundayHrs + PHHrs). Since
H 'Worked Hrs including OT' already INCLUDES overtime, adding I 'OT Hours'
separately double-counted OT, giving 255.02 instead of 252.07 for Kamlesh.

Fixed to =H+L+M (WorkedHrs incl OT + Sunday Hrs + PH Hrs).
Kamlesh now: 216.07 + 36 + 0 = 252.07 ✓ (matches Payroll Summary + HRMS UI)

Also regenerated all 3 Excel files from fresh production DB data after
pushing earlier fixes to GitHub/Vercel. All 3 now show consistent values:
- Present: 24, Absent: 3, Sundays: 4 → Total 31 days ✓
- Worked Hrs incl OT: 216:04
- Additional Hrs (Sundays): 36:00
- Total Hrs: 252:04
- Gross Salary: ₹17,166
</commit_message>
<xml_diff>
--- a/download/Payroll_Master_July_2026.xlsx
+++ b/download/Payroll_Master_July_2026.xlsx
@@ -3264,7 +3264,7 @@
         <v>0</v>
       </c>
       <c r="N5" s="17">
-        <f>H5+I5+L5+M5</f>
+        <f>H5+L5+M5</f>
         <v/>
       </c>
       <c r="O5" s="19">
@@ -3349,7 +3349,7 @@
         <v>0</v>
       </c>
       <c r="N6" s="24">
-        <f>H6+I6+L6+M6</f>
+        <f>H6+L6+M6</f>
         <v/>
       </c>
       <c r="O6" s="26">
@@ -3434,7 +3434,7 @@
         <v>0</v>
       </c>
       <c r="N7" s="17">
-        <f>H7+I7+L7+M7</f>
+        <f>H7+L7+M7</f>
         <v/>
       </c>
       <c r="O7" s="19">
@@ -3519,7 +3519,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="24">
-        <f>H8+I8+L8+M8</f>
+        <f>H8+L8+M8</f>
         <v/>
       </c>
       <c r="O8" s="26">
@@ -3604,7 +3604,7 @@
         <v>0</v>
       </c>
       <c r="N9" s="17">
-        <f>H9+I9+L9+M9</f>
+        <f>H9+L9+M9</f>
         <v/>
       </c>
       <c r="O9" s="19">
@@ -3689,7 +3689,7 @@
         <v>0</v>
       </c>
       <c r="N10" s="24">
-        <f>H10+I10+L10+M10</f>
+        <f>H10+L10+M10</f>
         <v/>
       </c>
       <c r="O10" s="26">
@@ -3774,7 +3774,7 @@
         <v>0</v>
       </c>
       <c r="N11" s="17">
-        <f>H11+I11+L11+M11</f>
+        <f>H11+L11+M11</f>
         <v/>
       </c>
       <c r="O11" s="19">
@@ -3859,7 +3859,7 @@
         <v>0</v>
       </c>
       <c r="N12" s="24">
-        <f>H12+I12+L12+M12</f>
+        <f>H12+L12+M12</f>
         <v/>
       </c>
       <c r="O12" s="26">
@@ -3944,7 +3944,7 @@
         <v>0</v>
       </c>
       <c r="N13" s="17">
-        <f>H13+I13+L13+M13</f>
+        <f>H13+L13+M13</f>
         <v/>
       </c>
       <c r="O13" s="19">
@@ -4029,7 +4029,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="24">
-        <f>H14+I14+L14+M14</f>
+        <f>H14+L14+M14</f>
         <v/>
       </c>
       <c r="O14" s="26">
@@ -4114,7 +4114,7 @@
         <v>0</v>
       </c>
       <c r="N15" s="17">
-        <f>H15+I15+L15+M15</f>
+        <f>H15+L15+M15</f>
         <v/>
       </c>
       <c r="O15" s="19">
@@ -4199,7 +4199,7 @@
         <v>0</v>
       </c>
       <c r="N16" s="24">
-        <f>H16+I16+L16+M16</f>
+        <f>H16+L16+M16</f>
         <v/>
       </c>
       <c r="O16" s="26">
@@ -4284,7 +4284,7 @@
         <v>0</v>
       </c>
       <c r="N17" s="17">
-        <f>H17+I17+L17+M17</f>
+        <f>H17+L17+M17</f>
         <v/>
       </c>
       <c r="O17" s="19">
@@ -4369,7 +4369,7 @@
         <v>0</v>
       </c>
       <c r="N18" s="24">
-        <f>H18+I18+L18+M18</f>
+        <f>H18+L18+M18</f>
         <v/>
       </c>
       <c r="O18" s="26">
@@ -4454,7 +4454,7 @@
         <v>0</v>
       </c>
       <c r="N19" s="17">
-        <f>H19+I19+L19+M19</f>
+        <f>H19+L19+M19</f>
         <v/>
       </c>
       <c r="O19" s="19">
@@ -4776,7 +4776,7 @@
         <v>0</v>
       </c>
       <c r="N5" s="17">
-        <f>H5+I5+L5+M5</f>
+        <f>H5+L5+M5</f>
         <v/>
       </c>
       <c r="O5" s="19">
@@ -4861,7 +4861,7 @@
         <v>0</v>
       </c>
       <c r="N6" s="24">
-        <f>H6+I6+L6+M6</f>
+        <f>H6+L6+M6</f>
         <v/>
       </c>
       <c r="O6" s="26">
@@ -4946,7 +4946,7 @@
         <v>0</v>
       </c>
       <c r="N7" s="17">
-        <f>H7+I7+L7+M7</f>
+        <f>H7+L7+M7</f>
         <v/>
       </c>
       <c r="O7" s="19">
@@ -5031,7 +5031,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="24">
-        <f>H8+I8+L8+M8</f>
+        <f>H8+L8+M8</f>
         <v/>
       </c>
       <c r="O8" s="26">
@@ -5116,7 +5116,7 @@
         <v>0</v>
       </c>
       <c r="N9" s="17">
-        <f>H9+I9+L9+M9</f>
+        <f>H9+L9+M9</f>
         <v/>
       </c>
       <c r="O9" s="19">
@@ -5201,7 +5201,7 @@
         <v>0</v>
       </c>
       <c r="N10" s="24">
-        <f>H10+I10+L10+M10</f>
+        <f>H10+L10+M10</f>
         <v/>
       </c>
       <c r="O10" s="26">
@@ -5286,7 +5286,7 @@
         <v>0</v>
       </c>
       <c r="N11" s="17">
-        <f>H11+I11+L11+M11</f>
+        <f>H11+L11+M11</f>
         <v/>
       </c>
       <c r="O11" s="19">
@@ -5371,7 +5371,7 @@
         <v>0</v>
       </c>
       <c r="N12" s="24">
-        <f>H12+I12+L12+M12</f>
+        <f>H12+L12+M12</f>
         <v/>
       </c>
       <c r="O12" s="26">
@@ -5456,7 +5456,7 @@
         <v>0</v>
       </c>
       <c r="N13" s="17">
-        <f>H13+I13+L13+M13</f>
+        <f>H13+L13+M13</f>
         <v/>
       </c>
       <c r="O13" s="19">
@@ -5541,7 +5541,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="24">
-        <f>H14+I14+L14+M14</f>
+        <f>H14+L14+M14</f>
         <v/>
       </c>
       <c r="O14" s="26">
@@ -5626,7 +5626,7 @@
         <v>0</v>
       </c>
       <c r="N15" s="17">
-        <f>H15+I15+L15+M15</f>
+        <f>H15+L15+M15</f>
         <v/>
       </c>
       <c r="O15" s="19">
@@ -5711,7 +5711,7 @@
         <v>0</v>
       </c>
       <c r="N16" s="24">
-        <f>H16+I16+L16+M16</f>
+        <f>H16+L16+M16</f>
         <v/>
       </c>
       <c r="O16" s="26">
@@ -5796,7 +5796,7 @@
         <v>0</v>
       </c>
       <c r="N17" s="17">
-        <f>H17+I17+L17+M17</f>
+        <f>H17+L17+M17</f>
         <v/>
       </c>
       <c r="O17" s="19">
@@ -5881,7 +5881,7 @@
         <v>0</v>
       </c>
       <c r="N18" s="24">
-        <f>H18+I18+L18+M18</f>
+        <f>H18+L18+M18</f>
         <v/>
       </c>
       <c r="O18" s="26">
@@ -5966,7 +5966,7 @@
         <v>0</v>
       </c>
       <c r="N19" s="17">
-        <f>H19+I19+L19+M19</f>
+        <f>H19+L19+M19</f>
         <v/>
       </c>
       <c r="O19" s="19">
@@ -6051,7 +6051,7 @@
         <v>0</v>
       </c>
       <c r="N20" s="24">
-        <f>H20+I20+L20+M20</f>
+        <f>H20+L20+M20</f>
         <v/>
       </c>
       <c r="O20" s="26">
@@ -6373,7 +6373,7 @@
         <v>0</v>
       </c>
       <c r="N5" s="17">
-        <f>H5+I5+L5+M5</f>
+        <f>H5+L5+M5</f>
         <v/>
       </c>
       <c r="O5" s="19">
@@ -6458,7 +6458,7 @@
         <v>0</v>
       </c>
       <c r="N6" s="24">
-        <f>H6+I6+L6+M6</f>
+        <f>H6+L6+M6</f>
         <v/>
       </c>
       <c r="O6" s="26">
@@ -6543,7 +6543,7 @@
         <v>0</v>
       </c>
       <c r="N7" s="17">
-        <f>H7+I7+L7+M7</f>
+        <f>H7+L7+M7</f>
         <v/>
       </c>
       <c r="O7" s="19">
@@ -6628,7 +6628,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="24">
-        <f>H8+I8+L8+M8</f>
+        <f>H8+L8+M8</f>
         <v/>
       </c>
       <c r="O8" s="26">
@@ -6713,7 +6713,7 @@
         <v>0</v>
       </c>
       <c r="N9" s="17">
-        <f>H9+I9+L9+M9</f>
+        <f>H9+L9+M9</f>
         <v/>
       </c>
       <c r="O9" s="19">
@@ -7035,7 +7035,7 @@
         <v>0</v>
       </c>
       <c r="N5" s="17">
-        <f>H5+I5+L5+M5</f>
+        <f>H5+L5+M5</f>
         <v/>
       </c>
       <c r="O5" s="19">
@@ -7120,7 +7120,7 @@
         <v>0</v>
       </c>
       <c r="N6" s="24">
-        <f>H6+I6+L6+M6</f>
+        <f>H6+L6+M6</f>
         <v/>
       </c>
       <c r="O6" s="26">
@@ -7205,7 +7205,7 @@
         <v>0</v>
       </c>
       <c r="N7" s="17">
-        <f>H7+I7+L7+M7</f>
+        <f>H7+L7+M7</f>
         <v/>
       </c>
       <c r="O7" s="19">
@@ -7290,7 +7290,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="24">
-        <f>H8+I8+L8+M8</f>
+        <f>H8+L8+M8</f>
         <v/>
       </c>
       <c r="O8" s="26">
@@ -7375,7 +7375,7 @@
         <v>0</v>
       </c>
       <c r="N9" s="17">
-        <f>H9+I9+L9+M9</f>
+        <f>H9+L9+M9</f>
         <v/>
       </c>
       <c r="O9" s="19">
@@ -7460,7 +7460,7 @@
         <v>0</v>
       </c>
       <c r="N10" s="24">
-        <f>H10+I10+L10+M10</f>
+        <f>H10+L10+M10</f>
         <v/>
       </c>
       <c r="O10" s="26">

</xml_diff>